<commit_message>
Switch to A$, add editable Weights sheet with round-trip persistence
- Currency changed throughout to A$
- New Weights sheet: rows=people, cols=expenses, value=split weight
  - 0.0 = excluded (grey), any positive = proportional share (green CF)
  - Pre-filled from EXPENSES splits config on first run
  - On re-runs, weights are read back from the existing Excel so
    edits survive without touching the Python file
- compute_splits() now takes a weights dict directly
- All other sheets (Splits, Balances, Settlement, WhatsApp) refresh
  from the read-back weights automatically

https://claude.ai/code/session_01KV4Tu2Dw8SUecueLZvfAaA
</commit_message>
<xml_diff>
--- a/HF_Weekend_Expense_Splitter.xlsx
+++ b/HF_Weekend_Expense_Splitter.xlsx
@@ -10,10 +10,11 @@
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Attendees" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Splits" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Balances" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settlement" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="WhatsApp" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Weights" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Splits" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Balances" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Settlement" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="WhatsApp" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,10 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="£#,##0.00"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;A$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0#"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,7 +39,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="20"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -70,6 +72,18 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00555555"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -190,17 +204,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ED7D31"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ED7D31"/>
       </patternFill>
     </fill>
     <fill>
@@ -232,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -268,9 +282,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -291,78 +302,109 @@
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="15" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DDDDDD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -724,156 +766,108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B23"/>
+  <dimension ref="B2:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2" ht="44" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>HF WEEKEND — EXPENSE SPLITTER</t>
+          <t>HF WEEKEND — EXPENSE SPLITTER  (A$)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated 19 Apr 2026  ·  16 attendees  ·  6 expenses  ·  Total £2,640.00</t>
+          <t>Generated 20 Apr 2026  ·  16 attendees  ·  6 expenses  ·  Total A$2,640.00</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>HOW TO USE THIS FILE</t>
+          <t>HOW TO USE</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>1.  Attendees sheet  — update the 16 names (Klaus and Louise already noted).</t>
+          <t>1.  Edit ATTENDEES &amp; EXPENSES in expense_splitter.py (names, amounts, who paid).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2.  Expenses sheet   — add/edit expense rows. One row per payment.</t>
+          <t>2.  Run script → Excel created with a pre-filled Weights sheet.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>3.  Splits sheet     — shows each person's share per expense (auto-calculated).</t>
+          <t>3.  Open Excel → go to the Weights sheet → enter each person's weight per expense.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>4.  Balances sheet   — net position for every attendee.</t>
+          <t>4.  Re-run script → weights are read back, everything else refreshes.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>5.  Settlement sheet — minimum payments to clear all debts.</t>
-        </is>
-      </c>
+      <c r="B10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>6.  WhatsApp sheet   — ready-to-paste message for the group.</t>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>WEIGHTS SHEET RULES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>7.  Re-run expense_splitter.py any time to refresh all calculations.</t>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  0.0  = person not included in that expense (grey cell)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="5" t="inlineStr"/>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1.0  = standard full share</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>SPLIT RULES FOR THIS WEEKEND</t>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  0.5  = half a standard share</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Standard expenses:     split evenly 16 ways</t>
+          <t xml:space="preserve">  Shares are proportional: e.g. ten 1.0s + two 0.5s → each 1.0 pays 1/11, each 0.5 pays 1/22</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Saturday Drinks:       Klaus gets a smaller share (~1/3 of standard)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Sunday Breakfast:      Klaus &amp; Louise not present → cost split 14 ways</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>ADDING MORE EXPENSES</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Add a row to the EXPENSES list in expense_splitter.py, then re-run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Use "splits": "even"  for a standard split.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Use "splits": {"PersonName": weight, "default": 1.0}  for custom splits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Weight 0 = person not included. Weight 0.3 = gets 30% of a standard share.</t>
+          <t xml:space="preserve">  To split evenly among N people: give each of those N people any equal weight (e.g. all 1.0)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -889,7 +883,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1104,7 +1098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1113,11 +1107,10 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
           <t>#</t>
@@ -1145,251 +1138,215 @@
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
-          <t>Amount (£)</t>
+          <t>Amount (A$)</t>
         </is>
       </c>
       <c r="G1" s="8" t="inlineStr">
         <is>
-          <t>Split Rule</t>
-        </is>
-      </c>
-      <c r="H1" s="15" t="inlineStr">
-        <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="A2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Accommodation</t>
         </is>
       </c>
-      <c r="D2" s="16" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>Accommodation</t>
         </is>
       </c>
-      <c r="E2" s="16" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="F2" s="17" t="n">
+      <c r="F2" s="16" t="n">
         <v>960</v>
       </c>
-      <c r="G2" s="16" t="inlineStr">
-        <is>
-          <t>Even (÷16)</t>
-        </is>
-      </c>
-      <c r="H2" s="18" t="inlineStr">
-        <is>
-          <t>Full weekend accommodation, all 16</t>
+      <c r="G2" s="17" t="inlineStr">
+        <is>
+          <t>Full weekend, all 16</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>Saturday Lunch</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>Food</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="F3" s="20" t="n">
+      <c r="F3" s="19" t="n">
         <v>240</v>
       </c>
-      <c r="G3" s="19" t="inlineStr">
-        <is>
-          <t>Even (÷16)</t>
-        </is>
-      </c>
-      <c r="H3" s="21" t="inlineStr"/>
+      <c r="G3" s="20" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="n">
+      <c r="A4" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C4" s="22" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Saturday Drinks</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Drinks</t>
         </is>
       </c>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Taylor</t>
         </is>
       </c>
-      <c r="F4" s="23" t="n">
+      <c r="F4" s="22" t="n">
         <v>320</v>
       </c>
-      <c r="G4" s="22" t="inlineStr">
-        <is>
-          <t>Custom — see Splits sheet</t>
-        </is>
-      </c>
-      <c r="H4" s="24" t="inlineStr">
-        <is>
-          <t>Klaus smaller share (approx ⅓ of standard portion)</t>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>Klaus smaller share (~1/3)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n">
+      <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Saturday Dinner</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Food</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Morgan</t>
         </is>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="19" t="n">
         <v>480</v>
       </c>
-      <c r="G5" s="19" t="inlineStr">
-        <is>
-          <t>Even (÷16)</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr"/>
+      <c r="G5" s="20" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n">
+      <c r="A6" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Sunday Breakfast</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Food</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Jamie</t>
         </is>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="19" t="n">
         <v>280</v>
       </c>
-      <c r="G6" s="19" t="inlineStr">
-        <is>
-          <t>Custom — see Splits sheet</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>Klaus &amp; Louise not present → split 14 ways</t>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Klaus &amp; Louise not present</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Sunday Lunch</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Food</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Casey</t>
         </is>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="19" t="n">
         <v>360</v>
       </c>
-      <c r="G7" s="19" t="inlineStr">
-        <is>
-          <t>Even (÷16)</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr"/>
+      <c r="G7" s="20" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="n"/>
-      <c r="B8" s="25" t="n"/>
-      <c r="C8" s="25" t="n"/>
-      <c r="D8" s="25" t="n"/>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="A8" s="24" t="n"/>
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="25" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="26" t="n">
         <v>2640</v>
       </c>
-      <c r="G8" s="25" t="n"/>
-      <c r="H8" s="25" t="n"/>
+      <c r="G8" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1402,124 +1359,659 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>SPLIT WEIGHTS — edit this sheet, then re-run expense_splitter.py to refresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>0.0 = excluded  |  1.0 = full share  |  0.5 = half share  |  Any positive number works — shares are proportional to weights in each column</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="B3" s="30" t="inlineStr">
+        <is>
+          <t>Fri: Accommodation</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="inlineStr">
+        <is>
+          <t>Sat: Saturday Lunch</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>Sat: Saturday Drinks</t>
+        </is>
+      </c>
+      <c r="E3" s="30" t="inlineStr">
+        <is>
+          <t>Sat: Saturday Dinner</t>
+        </is>
+      </c>
+      <c r="F3" s="30" t="inlineStr">
+        <is>
+          <t>Sun: Sunday Breakfast</t>
+        </is>
+      </c>
+      <c r="G3" s="30" t="inlineStr">
+        <is>
+          <t>Sun: Sunday Lunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Paid by →</t>
+        </is>
+      </c>
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>Alex  A$960</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="inlineStr">
+        <is>
+          <t>Sam  A$240</t>
+        </is>
+      </c>
+      <c r="D4" s="32" t="inlineStr">
+        <is>
+          <t>Taylor  A$320</t>
+        </is>
+      </c>
+      <c r="E4" s="32" t="inlineStr">
+        <is>
+          <t>Morgan  A$480</t>
+        </is>
+      </c>
+      <c r="F4" s="32" t="inlineStr">
+        <is>
+          <t>Jamie  A$280</t>
+        </is>
+      </c>
+      <c r="G4" s="32" t="inlineStr">
+        <is>
+          <t>Casey  A$360</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Klaus</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="34" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E5" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Louise</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B7" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Taylor</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Jamie</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Casey</t>
+        </is>
+      </c>
+      <c r="B13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>Riley</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>Drew</t>
+        </is>
+      </c>
+      <c r="B15" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>Quinn</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>Avery</t>
+        </is>
+      </c>
+      <c r="B17" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>Blake</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>Charlie</t>
+        </is>
+      </c>
+      <c r="B19" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>Dylan</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5:G20">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="30" t="inlineStr">
         <is>
           <t>Fri: Accommodation</t>
         </is>
       </c>
-      <c r="C1" s="28" t="inlineStr">
+      <c r="C1" s="30" t="inlineStr">
         <is>
           <t>Sat: Saturday Lunch</t>
         </is>
       </c>
-      <c r="D1" s="28" t="inlineStr">
+      <c r="D1" s="30" t="inlineStr">
         <is>
           <t>Sat: Saturday Drinks</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E1" s="30" t="inlineStr">
         <is>
           <t>Sat: Saturday Dinner</t>
         </is>
       </c>
-      <c r="F1" s="28" t="inlineStr">
+      <c r="F1" s="30" t="inlineStr">
         <is>
           <t>Sun: Sunday Breakfast</t>
         </is>
       </c>
-      <c r="G1" s="28" t="inlineStr">
+      <c r="G1" s="30" t="inlineStr">
         <is>
           <t>Sun: Sunday Lunch</t>
         </is>
       </c>
-      <c r="H1" s="29" t="inlineStr">
+      <c r="H1" s="38" t="inlineStr">
         <is>
           <t>Total Owed</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>Paid by:</t>
         </is>
       </c>
-      <c r="B2" s="31" t="inlineStr">
+      <c r="B2" s="32" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="C2" s="31" t="inlineStr">
+      <c r="C2" s="32" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="D2" s="31" t="inlineStr">
+      <c r="D2" s="32" t="inlineStr">
         <is>
           <t>Taylor</t>
         </is>
       </c>
-      <c r="E2" s="31" t="inlineStr">
+      <c r="E2" s="32" t="inlineStr">
         <is>
           <t>Morgan</t>
         </is>
       </c>
-      <c r="F2" s="31" t="inlineStr">
+      <c r="F2" s="32" t="inlineStr">
         <is>
           <t>Jamie</t>
         </is>
       </c>
-      <c r="G2" s="31" t="inlineStr">
+      <c r="G2" s="32" t="inlineStr">
         <is>
           <t>Casey</t>
         </is>
       </c>
-      <c r="H2" s="22" t="inlineStr"/>
+      <c r="H2" s="21" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="inlineStr">
-        <is>
-          <t>Total:</t>
-        </is>
-      </c>
-      <c r="B3" s="32" t="n">
-        <v>960</v>
-      </c>
-      <c r="C3" s="32" t="n">
-        <v>240</v>
-      </c>
-      <c r="D3" s="32" t="n">
-        <v>320</v>
-      </c>
-      <c r="E3" s="32" t="n">
-        <v>480</v>
-      </c>
-      <c r="F3" s="32" t="n">
-        <v>280</v>
-      </c>
-      <c r="G3" s="32" t="n">
-        <v>360</v>
-      </c>
-      <c r="H3" s="22" t="inlineStr"/>
+      <c r="A3" s="31" t="inlineStr">
+        <is>
+          <t>Amount:</t>
+        </is>
+      </c>
+      <c r="B3" s="32" t="inlineStr">
+        <is>
+          <t>A$960</t>
+        </is>
+      </c>
+      <c r="C3" s="32" t="inlineStr">
+        <is>
+          <t>A$240</t>
+        </is>
+      </c>
+      <c r="D3" s="32" t="inlineStr">
+        <is>
+          <t>A$320</t>
+        </is>
+      </c>
+      <c r="E3" s="32" t="inlineStr">
+        <is>
+          <t>A$480</t>
+        </is>
+      </c>
+      <c r="F3" s="32" t="inlineStr">
+        <is>
+          <t>A$280</t>
+        </is>
+      </c>
+      <c r="G3" s="32" t="inlineStr">
+        <is>
+          <t>A$360</t>
+        </is>
+      </c>
+      <c r="H3" s="21" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="33" t="inlineStr">
@@ -1527,27 +2019,27 @@
           <t>Klaus</t>
         </is>
       </c>
-      <c r="B4" s="34" t="n">
+      <c r="B4" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C4" s="34" t="n">
+      <c r="C4" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D4" s="34" t="n">
+      <c r="D4" s="39" t="n">
         <v>6.2</v>
       </c>
-      <c r="E4" s="34" t="n">
+      <c r="E4" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F4" s="35" t="inlineStr">
+      <c r="F4" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G4" s="34" t="n">
+      <c r="G4" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H4" s="36" t="n">
+      <c r="H4" s="41" t="n">
         <v>133.7</v>
       </c>
     </row>
@@ -1557,27 +2049,27 @@
           <t>Louise</t>
         </is>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="C5" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D5" s="37" t="n">
+      <c r="D5" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E5" s="37" t="n">
+      <c r="E5" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F5" s="35" t="inlineStr">
+      <c r="F5" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="37" t="n">
+      <c r="G5" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H5" s="36" t="n">
+      <c r="H5" s="41" t="n">
         <v>148.42</v>
       </c>
     </row>
@@ -1587,25 +2079,25 @@
           <t>Alex</t>
         </is>
       </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="39" t="n">
         <v>20.92</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G6" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H6" s="36" t="n">
+      <c r="H6" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1615,25 +2107,25 @@
           <t>Sam</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="C7" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="37" t="n">
+      <c r="D7" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="E7" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F7" s="37" t="n">
+      <c r="F7" s="42" t="n">
         <v>20</v>
       </c>
-      <c r="G7" s="37" t="n">
+      <c r="G7" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H7" s="36" t="n">
+      <c r="H7" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1643,25 +2135,25 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="B8" s="34" t="n">
+      <c r="B8" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="39" t="n">
         <v>20.92</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="34" t="n">
+      <c r="G8" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H8" s="36" t="n">
+      <c r="H8" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1671,25 +2163,25 @@
           <t>Taylor</t>
         </is>
       </c>
-      <c r="B9" s="37" t="n">
+      <c r="B9" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C9" s="37" t="n">
+      <c r="C9" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D9" s="37" t="n">
+      <c r="D9" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E9" s="37" t="n">
+      <c r="E9" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F9" s="37" t="n">
+      <c r="F9" s="42" t="n">
         <v>20</v>
       </c>
-      <c r="G9" s="37" t="n">
+      <c r="G9" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H9" s="36" t="n">
+      <c r="H9" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1699,25 +2191,25 @@
           <t>Morgan</t>
         </is>
       </c>
-      <c r="B10" s="34" t="n">
+      <c r="B10" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C10" s="34" t="n">
+      <c r="C10" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="39" t="n">
         <v>20.92</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G10" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H10" s="36" t="n">
+      <c r="H10" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1727,25 +2219,25 @@
           <t>Jamie</t>
         </is>
       </c>
-      <c r="B11" s="37" t="n">
+      <c r="B11" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C11" s="37" t="n">
+      <c r="C11" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D11" s="37" t="n">
+      <c r="D11" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E11" s="37" t="n">
+      <c r="E11" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F11" s="37" t="n">
+      <c r="F11" s="42" t="n">
         <v>20</v>
       </c>
-      <c r="G11" s="37" t="n">
+      <c r="G11" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H11" s="36" t="n">
+      <c r="H11" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1755,25 +2247,25 @@
           <t>Casey</t>
         </is>
       </c>
-      <c r="B12" s="34" t="n">
+      <c r="B12" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C12" s="34" t="n">
+      <c r="C12" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="39" t="n">
         <v>20.92</v>
       </c>
-      <c r="E12" s="34" t="n">
+      <c r="E12" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="G12" s="34" t="n">
+      <c r="G12" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H12" s="36" t="n">
+      <c r="H12" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1783,25 +2275,25 @@
           <t>Riley</t>
         </is>
       </c>
-      <c r="B13" s="37" t="n">
+      <c r="B13" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C13" s="37" t="n">
+      <c r="C13" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D13" s="37" t="n">
+      <c r="D13" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E13" s="37" t="n">
+      <c r="E13" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F13" s="37" t="n">
+      <c r="F13" s="42" t="n">
         <v>20</v>
       </c>
-      <c r="G13" s="37" t="n">
+      <c r="G13" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H13" s="36" t="n">
+      <c r="H13" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1811,25 +2303,25 @@
           <t>Drew</t>
         </is>
       </c>
-      <c r="B14" s="34" t="n">
+      <c r="B14" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C14" s="34" t="n">
+      <c r="C14" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D14" s="34" t="n">
+      <c r="D14" s="39" t="n">
         <v>20.92</v>
       </c>
-      <c r="E14" s="34" t="n">
+      <c r="E14" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F14" s="34" t="n">
+      <c r="F14" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="G14" s="34" t="n">
+      <c r="G14" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H14" s="36" t="n">
+      <c r="H14" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1839,25 +2331,25 @@
           <t>Quinn</t>
         </is>
       </c>
-      <c r="B15" s="37" t="n">
+      <c r="B15" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C15" s="37" t="n">
+      <c r="C15" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D15" s="37" t="n">
+      <c r="D15" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E15" s="37" t="n">
+      <c r="E15" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F15" s="37" t="n">
+      <c r="F15" s="42" t="n">
         <v>20</v>
       </c>
-      <c r="G15" s="37" t="n">
+      <c r="G15" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H15" s="36" t="n">
+      <c r="H15" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1867,25 +2359,25 @@
           <t>Avery</t>
         </is>
       </c>
-      <c r="B16" s="34" t="n">
+      <c r="B16" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C16" s="34" t="n">
+      <c r="C16" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D16" s="34" t="n">
+      <c r="D16" s="39" t="n">
         <v>20.92</v>
       </c>
-      <c r="E16" s="34" t="n">
+      <c r="E16" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F16" s="34" t="n">
+      <c r="F16" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="G16" s="34" t="n">
+      <c r="G16" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H16" s="36" t="n">
+      <c r="H16" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1895,25 +2387,25 @@
           <t>Blake</t>
         </is>
       </c>
-      <c r="B17" s="37" t="n">
+      <c r="B17" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C17" s="37" t="n">
+      <c r="C17" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D17" s="37" t="n">
+      <c r="D17" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E17" s="37" t="n">
+      <c r="E17" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F17" s="37" t="n">
+      <c r="F17" s="42" t="n">
         <v>20</v>
       </c>
-      <c r="G17" s="37" t="n">
+      <c r="G17" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H17" s="36" t="n">
+      <c r="H17" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1923,25 +2415,25 @@
           <t>Charlie</t>
         </is>
       </c>
-      <c r="B18" s="34" t="n">
+      <c r="B18" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C18" s="34" t="n">
+      <c r="C18" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="D18" s="34" t="n">
+      <c r="D18" s="39" t="n">
         <v>20.92</v>
       </c>
-      <c r="E18" s="34" t="n">
+      <c r="E18" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="F18" s="34" t="n">
+      <c r="F18" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="G18" s="34" t="n">
+      <c r="G18" s="39" t="n">
         <v>22.5</v>
       </c>
-      <c r="H18" s="36" t="n">
+      <c r="H18" s="41" t="n">
         <v>168.42</v>
       </c>
     </row>
@@ -1951,54 +2443,26 @@
           <t>Dylan</t>
         </is>
       </c>
-      <c r="B19" s="37" t="n">
+      <c r="B19" s="42" t="n">
         <v>60</v>
       </c>
-      <c r="C19" s="37" t="n">
+      <c r="C19" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="D19" s="37" t="n">
+      <c r="D19" s="42" t="n">
         <v>20.92</v>
       </c>
-      <c r="E19" s="37" t="n">
+      <c r="E19" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="F19" s="37" t="n">
+      <c r="F19" s="42" t="n">
         <v>20</v>
       </c>
-      <c r="G19" s="37" t="n">
+      <c r="G19" s="42" t="n">
         <v>22.5</v>
       </c>
-      <c r="H19" s="36" t="n">
+      <c r="H19" s="41" t="n">
         <v>168.42</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="26" t="inlineStr">
-        <is>
-          <t>Col Total (check)</t>
-        </is>
-      </c>
-      <c r="B20" s="27" t="n">
-        <v>960</v>
-      </c>
-      <c r="C20" s="27" t="n">
-        <v>240</v>
-      </c>
-      <c r="D20" s="27" t="n">
-        <v>320</v>
-      </c>
-      <c r="E20" s="27" t="n">
-        <v>480</v>
-      </c>
-      <c r="F20" s="27" t="n">
-        <v>280</v>
-      </c>
-      <c r="G20" s="27" t="n">
-        <v>360</v>
-      </c>
-      <c r="H20" s="38" t="n">
-        <v>2640</v>
       </c>
     </row>
   </sheetData>
@@ -2006,7 +2470,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2030,17 +2494,17 @@
       </c>
       <c r="B1" s="8" t="inlineStr">
         <is>
-          <t>Total Paid (£)</t>
+          <t>Total Paid (A$)</t>
         </is>
       </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
-          <t>Total Share (£)</t>
+          <t>Total Share (A$)</t>
         </is>
       </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>Net Balance (£)</t>
+          <t>Net Balance (A$)</t>
         </is>
       </c>
       <c r="E1" s="8" t="inlineStr">
@@ -2055,18 +2519,18 @@
           <t>Alex</t>
         </is>
       </c>
-      <c r="B2" s="37" t="n">
+      <c r="B2" s="42" t="n">
         <v>960</v>
       </c>
-      <c r="C2" s="37" t="n">
+      <c r="C2" s="42" t="n">
         <v>168.42</v>
       </c>
-      <c r="D2" s="39" t="n">
+      <c r="D2" s="43" t="n">
         <v>791.58</v>
       </c>
-      <c r="E2" s="40" t="inlineStr">
-        <is>
-          <t>Gets back £791.58</t>
+      <c r="E2" s="44" t="inlineStr">
+        <is>
+          <t>Gets back A$791.58</t>
         </is>
       </c>
     </row>
@@ -2076,18 +2540,18 @@
           <t>Morgan</t>
         </is>
       </c>
-      <c r="B3" s="34" t="n">
+      <c r="B3" s="39" t="n">
         <v>480</v>
       </c>
-      <c r="C3" s="34" t="n">
+      <c r="C3" s="39" t="n">
         <v>168.42</v>
       </c>
-      <c r="D3" s="39" t="n">
+      <c r="D3" s="43" t="n">
         <v>311.58</v>
       </c>
-      <c r="E3" s="40" t="inlineStr">
-        <is>
-          <t>Gets back £311.58</t>
+      <c r="E3" s="44" t="inlineStr">
+        <is>
+          <t>Gets back A$311.58</t>
         </is>
       </c>
     </row>
@@ -2097,18 +2561,18 @@
           <t>Casey</t>
         </is>
       </c>
-      <c r="B4" s="37" t="n">
+      <c r="B4" s="42" t="n">
         <v>360</v>
       </c>
-      <c r="C4" s="37" t="n">
+      <c r="C4" s="42" t="n">
         <v>168.42</v>
       </c>
-      <c r="D4" s="39" t="n">
+      <c r="D4" s="43" t="n">
         <v>191.58</v>
       </c>
-      <c r="E4" s="40" t="inlineStr">
-        <is>
-          <t>Gets back £191.58</t>
+      <c r="E4" s="44" t="inlineStr">
+        <is>
+          <t>Gets back A$191.58</t>
         </is>
       </c>
     </row>
@@ -2118,18 +2582,18 @@
           <t>Taylor</t>
         </is>
       </c>
-      <c r="B5" s="34" t="n">
+      <c r="B5" s="39" t="n">
         <v>320</v>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="C5" s="39" t="n">
         <v>168.42</v>
       </c>
-      <c r="D5" s="39" t="n">
+      <c r="D5" s="43" t="n">
         <v>151.58</v>
       </c>
-      <c r="E5" s="40" t="inlineStr">
-        <is>
-          <t>Gets back £151.58</t>
+      <c r="E5" s="44" t="inlineStr">
+        <is>
+          <t>Gets back A$151.58</t>
         </is>
       </c>
     </row>
@@ -2139,18 +2603,18 @@
           <t>Jamie</t>
         </is>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="42" t="n">
         <v>280</v>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="C6" s="42" t="n">
         <v>168.42</v>
       </c>
-      <c r="D6" s="39" t="n">
+      <c r="D6" s="43" t="n">
         <v>111.58</v>
       </c>
-      <c r="E6" s="40" t="inlineStr">
-        <is>
-          <t>Gets back £111.58</t>
+      <c r="E6" s="44" t="inlineStr">
+        <is>
+          <t>Gets back A$111.58</t>
         </is>
       </c>
     </row>
@@ -2160,18 +2624,18 @@
           <t>Sam</t>
         </is>
       </c>
-      <c r="B7" s="34" t="n">
+      <c r="B7" s="39" t="n">
         <v>240</v>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="C7" s="39" t="n">
         <v>168.42</v>
       </c>
-      <c r="D7" s="39" t="n">
+      <c r="D7" s="43" t="n">
         <v>71.58</v>
       </c>
-      <c r="E7" s="40" t="inlineStr">
-        <is>
-          <t>Gets back £71.58</t>
+      <c r="E7" s="44" t="inlineStr">
+        <is>
+          <t>Gets back A$71.58</t>
         </is>
       </c>
     </row>
@@ -2181,18 +2645,18 @@
           <t>Klaus</t>
         </is>
       </c>
-      <c r="B8" s="37" t="n">
+      <c r="B8" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="C8" s="42" t="n">
         <v>133.7</v>
       </c>
-      <c r="D8" s="41" t="n">
+      <c r="D8" s="45" t="n">
         <v>-133.7</v>
       </c>
-      <c r="E8" s="42" t="inlineStr">
-        <is>
-          <t>Owes £133.70</t>
+      <c r="E8" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$133.70</t>
         </is>
       </c>
     </row>
@@ -2202,18 +2666,18 @@
           <t>Louise</t>
         </is>
       </c>
-      <c r="B9" s="34" t="n">
+      <c r="B9" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="C9" s="39" t="n">
         <v>148.42</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D9" s="45" t="n">
         <v>-148.42</v>
       </c>
-      <c r="E9" s="42" t="inlineStr">
-        <is>
-          <t>Owes £148.42</t>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$148.42</t>
         </is>
       </c>
     </row>
@@ -2223,18 +2687,18 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="B10" s="37" t="n">
+      <c r="B10" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="37" t="n">
+      <c r="C10" s="42" t="n">
         <v>168.42</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D10" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E10" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
@@ -2244,18 +2708,18 @@
           <t>Riley</t>
         </is>
       </c>
-      <c r="B11" s="34" t="n">
+      <c r="B11" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="34" t="n">
+      <c r="C11" s="39" t="n">
         <v>168.42</v>
       </c>
-      <c r="D11" s="41" t="n">
+      <c r="D11" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E11" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
@@ -2265,18 +2729,18 @@
           <t>Drew</t>
         </is>
       </c>
-      <c r="B12" s="37" t="n">
+      <c r="B12" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="37" t="n">
+      <c r="C12" s="42" t="n">
         <v>168.42</v>
       </c>
-      <c r="D12" s="41" t="n">
+      <c r="D12" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E12" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
@@ -2286,18 +2750,18 @@
           <t>Quinn</t>
         </is>
       </c>
-      <c r="B13" s="34" t="n">
+      <c r="B13" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="34" t="n">
+      <c r="C13" s="39" t="n">
         <v>168.42</v>
       </c>
-      <c r="D13" s="41" t="n">
+      <c r="D13" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E13" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
@@ -2307,18 +2771,18 @@
           <t>Avery</t>
         </is>
       </c>
-      <c r="B14" s="37" t="n">
+      <c r="B14" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="37" t="n">
+      <c r="C14" s="42" t="n">
         <v>168.42</v>
       </c>
-      <c r="D14" s="41" t="n">
+      <c r="D14" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E14" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
@@ -2328,18 +2792,18 @@
           <t>Blake</t>
         </is>
       </c>
-      <c r="B15" s="34" t="n">
+      <c r="B15" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C15" s="39" t="n">
         <v>168.42</v>
       </c>
-      <c r="D15" s="41" t="n">
+      <c r="D15" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E15" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E15" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
@@ -2349,18 +2813,18 @@
           <t>Charlie</t>
         </is>
       </c>
-      <c r="B16" s="37" t="n">
+      <c r="B16" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="37" t="n">
+      <c r="C16" s="42" t="n">
         <v>168.42</v>
       </c>
-      <c r="D16" s="41" t="n">
+      <c r="D16" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E16" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E16" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
@@ -2370,44 +2834,44 @@
           <t>Dylan</t>
         </is>
       </c>
-      <c r="B17" s="34" t="n">
+      <c r="B17" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="34" t="n">
+      <c r="C17" s="39" t="n">
         <v>168.42</v>
       </c>
-      <c r="D17" s="41" t="n">
+      <c r="D17" s="45" t="n">
         <v>-168.42</v>
       </c>
-      <c r="E17" s="42" t="inlineStr">
-        <is>
-          <t>Owes £168.42</t>
+      <c r="E17" s="46" t="inlineStr">
+        <is>
+          <t>Owes A$168.42</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="27" t="n">
+      <c r="B18" s="26" t="n">
         <v>2640</v>
       </c>
-      <c r="C18" s="27" t="n">
+      <c r="C18" s="26" t="n">
         <v>2640</v>
       </c>
-      <c r="D18" s="27" t="n">
+      <c r="D18" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="25" t="n"/>
+      <c r="E18" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2422,50 +2886,50 @@
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="43" t="inlineStr">
+      <c r="B2" s="47" t="inlineStr">
         <is>
           <t>Recommended Settlement Plan — Minimum Transactions</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="B3" s="44" t="inlineStr">
-        <is>
-          <t>15 payment(s) required to fully settle all debts</t>
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>15 payment(s) to fully settle all debts</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="45" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C5" s="45" t="inlineStr">
+      <c r="C5" s="49" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="D5" s="45" t="inlineStr">
+      <c r="D5" s="49" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E5" s="45" t="inlineStr">
+      <c r="E5" s="49" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="F5" s="45" t="inlineStr">
-        <is>
-          <t>Amount (£)</t>
-        </is>
-      </c>
-      <c r="G5" s="45" t="inlineStr">
+      <c r="F5" s="49" t="inlineStr">
+        <is>
+          <t>Amount (A$)</t>
+        </is>
+      </c>
+      <c r="G5" s="49" t="inlineStr">
         <is>
           <t>Bank ref</t>
         </is>
@@ -2475,25 +2939,25 @@
       <c r="B6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="46" t="inlineStr">
+      <c r="C6" s="50" t="inlineStr">
         <is>
           <t>Riley</t>
         </is>
       </c>
-      <c r="D6" s="47" t="inlineStr">
+      <c r="D6" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="50" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="F6" s="48" t="n">
+      <c r="F6" s="52" t="n">
         <v>168.42</v>
       </c>
-      <c r="G6" s="49" t="inlineStr">
+      <c r="G6" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Riley</t>
         </is>
@@ -2503,25 +2967,25 @@
       <c r="B7" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="50" t="inlineStr">
+      <c r="C7" s="54" t="inlineStr">
         <is>
           <t>Quinn</t>
         </is>
       </c>
-      <c r="D7" s="51" t="inlineStr">
+      <c r="D7" s="55" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E7" s="50" t="inlineStr">
+      <c r="E7" s="54" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="F7" s="52" t="n">
+      <c r="F7" s="56" t="n">
         <v>168.42</v>
       </c>
-      <c r="G7" s="53" t="inlineStr">
+      <c r="G7" s="57" t="inlineStr">
         <is>
           <t>HF Weekend Quinn</t>
         </is>
@@ -2531,25 +2995,25 @@
       <c r="B8" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="46" t="inlineStr">
+      <c r="C8" s="50" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D8" s="47" t="inlineStr">
+      <c r="D8" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E8" s="46" t="inlineStr">
+      <c r="E8" s="50" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="F8" s="48" t="n">
+      <c r="F8" s="52" t="n">
         <v>168.42</v>
       </c>
-      <c r="G8" s="49" t="inlineStr">
+      <c r="G8" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Jordan</t>
         </is>
@@ -2559,25 +3023,25 @@
       <c r="B9" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="50" t="inlineStr">
+      <c r="C9" s="54" t="inlineStr">
         <is>
           <t>Dylan</t>
         </is>
       </c>
-      <c r="D9" s="51" t="inlineStr">
+      <c r="D9" s="55" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E9" s="50" t="inlineStr">
+      <c r="E9" s="54" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="F9" s="52" t="n">
+      <c r="F9" s="56" t="n">
         <v>168.42</v>
       </c>
-      <c r="G9" s="53" t="inlineStr">
+      <c r="G9" s="57" t="inlineStr">
         <is>
           <t>HF Weekend Dylan</t>
         </is>
@@ -2587,25 +3051,25 @@
       <c r="B10" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="46" t="inlineStr">
+      <c r="C10" s="50" t="inlineStr">
         <is>
           <t>Drew</t>
         </is>
       </c>
-      <c r="D10" s="47" t="inlineStr">
+      <c r="D10" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E10" s="46" t="inlineStr">
+      <c r="E10" s="50" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="F10" s="48" t="n">
+      <c r="F10" s="52" t="n">
         <v>117.9</v>
       </c>
-      <c r="G10" s="49" t="inlineStr">
+      <c r="G10" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Drew</t>
         </is>
@@ -2615,25 +3079,25 @@
       <c r="B11" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="C11" s="50" t="inlineStr">
+      <c r="C11" s="54" t="inlineStr">
         <is>
           <t>Drew</t>
         </is>
       </c>
-      <c r="D11" s="51" t="inlineStr">
+      <c r="D11" s="55" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E11" s="50" t="inlineStr">
+      <c r="E11" s="54" t="inlineStr">
         <is>
           <t>Morgan</t>
         </is>
       </c>
-      <c r="F11" s="52" t="n">
+      <c r="F11" s="56" t="n">
         <v>50.52</v>
       </c>
-      <c r="G11" s="53" t="inlineStr">
+      <c r="G11" s="57" t="inlineStr">
         <is>
           <t>HF Weekend Drew</t>
         </is>
@@ -2643,25 +3107,25 @@
       <c r="B12" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="50" t="inlineStr">
         <is>
           <t>Charlie</t>
         </is>
       </c>
-      <c r="D12" s="47" t="inlineStr">
+      <c r="D12" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E12" s="46" t="inlineStr">
+      <c r="E12" s="50" t="inlineStr">
         <is>
           <t>Morgan</t>
         </is>
       </c>
-      <c r="F12" s="48" t="n">
+      <c r="F12" s="52" t="n">
         <v>168.42</v>
       </c>
-      <c r="G12" s="49" t="inlineStr">
+      <c r="G12" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Charlie</t>
         </is>
@@ -2671,25 +3135,25 @@
       <c r="B13" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="C13" s="50" t="inlineStr">
+      <c r="C13" s="54" t="inlineStr">
         <is>
           <t>Blake</t>
         </is>
       </c>
-      <c r="D13" s="51" t="inlineStr">
+      <c r="D13" s="55" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E13" s="50" t="inlineStr">
+      <c r="E13" s="54" t="inlineStr">
         <is>
           <t>Morgan</t>
         </is>
       </c>
-      <c r="F13" s="52" t="n">
+      <c r="F13" s="56" t="n">
         <v>92.64</v>
       </c>
-      <c r="G13" s="53" t="inlineStr">
+      <c r="G13" s="57" t="inlineStr">
         <is>
           <t>HF Weekend Blake</t>
         </is>
@@ -2699,25 +3163,25 @@
       <c r="B14" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="C14" s="46" t="inlineStr">
+      <c r="C14" s="50" t="inlineStr">
         <is>
           <t>Blake</t>
         </is>
       </c>
-      <c r="D14" s="47" t="inlineStr">
+      <c r="D14" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E14" s="46" t="inlineStr">
+      <c r="E14" s="50" t="inlineStr">
         <is>
           <t>Casey</t>
         </is>
       </c>
-      <c r="F14" s="48" t="n">
+      <c r="F14" s="52" t="n">
         <v>75.78</v>
       </c>
-      <c r="G14" s="49" t="inlineStr">
+      <c r="G14" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Blake</t>
         </is>
@@ -2727,25 +3191,25 @@
       <c r="B15" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="C15" s="50" t="inlineStr">
+      <c r="C15" s="54" t="inlineStr">
         <is>
           <t>Avery</t>
         </is>
       </c>
-      <c r="D15" s="51" t="inlineStr">
+      <c r="D15" s="55" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E15" s="50" t="inlineStr">
+      <c r="E15" s="54" t="inlineStr">
         <is>
           <t>Casey</t>
         </is>
       </c>
-      <c r="F15" s="52" t="n">
+      <c r="F15" s="56" t="n">
         <v>115.8</v>
       </c>
-      <c r="G15" s="53" t="inlineStr">
+      <c r="G15" s="57" t="inlineStr">
         <is>
           <t>HF Weekend Avery</t>
         </is>
@@ -2755,25 +3219,25 @@
       <c r="B16" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="C16" s="46" t="inlineStr">
+      <c r="C16" s="50" t="inlineStr">
         <is>
           <t>Avery</t>
         </is>
       </c>
-      <c r="D16" s="47" t="inlineStr">
+      <c r="D16" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E16" s="46" t="inlineStr">
+      <c r="E16" s="50" t="inlineStr">
         <is>
           <t>Taylor</t>
         </is>
       </c>
-      <c r="F16" s="48" t="n">
+      <c r="F16" s="52" t="n">
         <v>52.62</v>
       </c>
-      <c r="G16" s="49" t="inlineStr">
+      <c r="G16" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Avery</t>
         </is>
@@ -2783,25 +3247,25 @@
       <c r="B17" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C17" s="50" t="inlineStr">
+      <c r="C17" s="54" t="inlineStr">
         <is>
           <t>Louise</t>
         </is>
       </c>
-      <c r="D17" s="51" t="inlineStr">
+      <c r="D17" s="55" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E17" s="50" t="inlineStr">
+      <c r="E17" s="54" t="inlineStr">
         <is>
           <t>Taylor</t>
         </is>
       </c>
-      <c r="F17" s="52" t="n">
+      <c r="F17" s="56" t="n">
         <v>98.95999999999999</v>
       </c>
-      <c r="G17" s="53" t="inlineStr">
+      <c r="G17" s="57" t="inlineStr">
         <is>
           <t>HF Weekend Louise</t>
         </is>
@@ -2811,25 +3275,25 @@
       <c r="B18" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="C18" s="46" t="inlineStr">
+      <c r="C18" s="50" t="inlineStr">
         <is>
           <t>Louise</t>
         </is>
       </c>
-      <c r="D18" s="47" t="inlineStr">
+      <c r="D18" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E18" s="46" t="inlineStr">
+      <c r="E18" s="50" t="inlineStr">
         <is>
           <t>Jamie</t>
         </is>
       </c>
-      <c r="F18" s="48" t="n">
+      <c r="F18" s="52" t="n">
         <v>49.46</v>
       </c>
-      <c r="G18" s="49" t="inlineStr">
+      <c r="G18" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Louise</t>
         </is>
@@ -2839,25 +3303,25 @@
       <c r="B19" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="C19" s="50" t="inlineStr">
+      <c r="C19" s="54" t="inlineStr">
         <is>
           <t>Klaus</t>
         </is>
       </c>
-      <c r="D19" s="51" t="inlineStr">
+      <c r="D19" s="55" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E19" s="50" t="inlineStr">
+      <c r="E19" s="54" t="inlineStr">
         <is>
           <t>Jamie</t>
         </is>
       </c>
-      <c r="F19" s="52" t="n">
+      <c r="F19" s="56" t="n">
         <v>62.12</v>
       </c>
-      <c r="G19" s="53" t="inlineStr">
+      <c r="G19" s="57" t="inlineStr">
         <is>
           <t>HF Weekend Klaus</t>
         </is>
@@ -2867,25 +3331,25 @@
       <c r="B20" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="46" t="inlineStr">
+      <c r="C20" s="50" t="inlineStr">
         <is>
           <t>Klaus</t>
         </is>
       </c>
-      <c r="D20" s="47" t="inlineStr">
+      <c r="D20" s="51" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="E20" s="46" t="inlineStr">
+      <c r="E20" s="50" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="F20" s="48" t="n">
+      <c r="F20" s="52" t="n">
         <v>71.58</v>
       </c>
-      <c r="G20" s="49" t="inlineStr">
+      <c r="G20" s="53" t="inlineStr">
         <is>
           <t>HF Weekend Klaus</t>
         </is>
@@ -2900,311 +3364,304 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B82"/>
+  <dimension ref="B1:B81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="B1" s="8" t="inlineStr">
         <is>
-          <t>WhatsApp Message  —  copy the yellow cell below and paste into your chat</t>
+          <t>WhatsApp Message  —  copy the yellow block below and paste into your chat</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="B2" s="54" t="inlineStr">
+      <c r="B2" s="58" t="inlineStr">
         <is>
           <t>─────────────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="B3" s="54" t="inlineStr">
+      <c r="B3" s="58" t="inlineStr">
         <is>
           <t>HF WEEKEND — EXPENSES &amp; SETTLEMENT</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="B4" s="54" t="inlineStr">
+      <c r="B4" s="58" t="inlineStr">
         <is>
           <t>─────────────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="B5" s="54" t="inlineStr"/>
+      <c r="B5" s="58" t="inlineStr"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="B6" s="54" t="inlineStr">
-        <is>
-          <t>Total spend: £2,640.00  |  16 people</t>
+      <c r="B6" s="58" t="inlineStr">
+        <is>
+          <t>Total spend: A$2,640.00  |  16 people</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="B7" s="54" t="inlineStr"/>
+      <c r="B7" s="58" t="inlineStr"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="B8" s="54" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>Expenses:</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Fri  Accommodation          £  960.00  (paid by Alex)</t>
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fri  Accommodation          A$  960.00  (paid by Alex)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="B10" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sat  Saturday Lunch         £  240.00  (paid by Sam)</t>
+      <c r="B10" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sat  Saturday Lunch         A$  240.00  (paid by Sam)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="B11" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sat  Saturday Drinks        £  320.00  (paid by Taylor)</t>
+      <c r="B11" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sat  Saturday Drinks        A$  320.00  (paid by Taylor)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sat  Saturday Dinner        £  480.00  (paid by Morgan)</t>
+      <c r="B12" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sat  Saturday Dinner        A$  480.00  (paid by Morgan)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sun  Sunday Breakfast       £  280.00  (paid by Jamie)</t>
+      <c r="B13" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sun  Sunday Breakfast       A$  280.00  (paid by Jamie)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sun  Sunday Lunch           £  360.00  (paid by Casey)</t>
+      <c r="B14" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sun  Sunday Lunch           A$  360.00  (paid by Casey)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="B15" s="54" t="inlineStr"/>
+      <c r="B15" s="58" t="inlineStr"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="B16" s="54" t="inlineStr">
+      <c r="B16" s="58" t="inlineStr">
         <is>
           <t>Split adjustments:</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="B17" s="54" t="inlineStr">
+      <c r="B17" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Sat Drinks: Klaus had a small share (~1/3 of standard)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="B18" s="54" t="inlineStr">
+      <c r="B18" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Sun Breakfast: Klaus &amp; Louise not present — split 14 ways</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="B19" s="54" t="inlineStr"/>
+      <c r="B19" s="58" t="inlineStr"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="54" t="inlineStr">
+      <c r="B20" s="58" t="inlineStr">
         <is>
           <t>Payments needed:</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="B21" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Riley pays Alex: £168.42</t>
+      <c r="B21" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Riley pays Alex: A$168.42</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="B22" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Quinn pays Alex: £168.42</t>
+      <c r="B22" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Quinn pays Alex: A$168.42</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="B23" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Jordan pays Alex: £168.42</t>
+      <c r="B23" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Jordan pays Alex: A$168.42</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="B24" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Dylan pays Alex: £168.42</t>
+      <c r="B24" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Dylan pays Alex: A$168.42</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="B25" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Drew pays Alex: £117.90</t>
+      <c r="B25" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Drew pays Alex: A$117.90</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="B26" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Drew pays Morgan: £50.52</t>
+      <c r="B26" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Drew pays Morgan: A$50.52</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="B27" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Charlie pays Morgan: £168.42</t>
+      <c r="B27" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Charlie pays Morgan: A$168.42</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Blake pays Morgan: £92.64</t>
+      <c r="B28" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blake pays Morgan: A$92.64</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Blake pays Casey: £75.78</t>
+      <c r="B29" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blake pays Casey: A$75.78</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="B30" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Avery pays Casey: £115.80</t>
+      <c r="B30" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Avery pays Casey: A$115.80</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="B31" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Avery pays Taylor: £52.62</t>
+      <c r="B31" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Avery pays Taylor: A$52.62</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Louise pays Taylor: £98.96</t>
+      <c r="B32" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Louise pays Taylor: A$98.96</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Louise pays Jamie: £49.46</t>
+      <c r="B33" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Louise pays Jamie: A$49.46</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Klaus pays Jamie: £62.12</t>
+      <c r="B34" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Klaus pays Jamie: A$62.12</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Klaus pays Sam: £71.58</t>
+      <c r="B35" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Klaus pays Sam: A$71.58</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="B36" s="54" t="inlineStr"/>
+      <c r="B36" s="58" t="inlineStr"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="B37" s="54" t="inlineStr">
-        <is>
-          <t>Please pay by bank transfer.</t>
+      <c r="B37" s="58" t="inlineStr">
+        <is>
+          <t>Please pay by bank transfer. Use your name as the reference.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="B38" s="54" t="inlineStr">
-        <is>
-          <t>Use your name as the reference.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="B39" s="54" t="inlineStr">
+      <c r="B38" s="58" t="inlineStr">
         <is>
           <t>─────────────────────────────────</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1">
-      <c r="B42" s="55" t="inlineStr">
+    <row r="41" ht="15" customHeight="1">
+      <c r="B41" s="59" t="inlineStr">
         <is>
           <t>─────────────────────────────────
 HF WEEKEND — EXPENSES &amp; SETTLEMENT
 ─────────────────────────────────
-Total spend: £2,640.00  |  16 people
+Total spend: A$2,640.00  |  16 people
 Expenses:
-  Fri  Accommodation          £  960.00  (paid by Alex)
-  Sat  Saturday Lunch         £  240.00  (paid by Sam)
-  Sat  Saturday Drinks        £  320.00  (paid by Taylor)
-  Sat  Saturday Dinner        £  480.00  (paid by Morgan)
-  Sun  Sunday Breakfast       £  280.00  (paid by Jamie)
-  Sun  Sunday Lunch           £  360.00  (paid by Casey)
+  Fri  Accommodation          A$  960.00  (paid by Alex)
+  Sat  Saturday Lunch         A$  240.00  (paid by Sam)
+  Sat  Saturday Drinks        A$  320.00  (paid by Taylor)
+  Sat  Saturday Dinner        A$  480.00  (paid by Morgan)
+  Sun  Sunday Breakfast       A$  280.00  (paid by Jamie)
+  Sun  Sunday Lunch           A$  360.00  (paid by Casey)
 Split adjustments:
   • Sat Drinks: Klaus had a small share (~1/3 of standard)
   • Sun Breakfast: Klaus &amp; Louise not present — split 14 ways
 Payments needed:
-  Riley pays Alex: £168.42
-  Quinn pays Alex: £168.42
-  Jordan pays Alex: £168.42
-  Dylan pays Alex: £168.42
-  Drew pays Alex: £117.90
-  Drew pays Morgan: £50.52
-  Charlie pays Morgan: £168.42
-  Blake pays Morgan: £92.64
-  Blake pays Casey: £75.78
-  Avery pays Casey: £115.80
-  Avery pays Taylor: £52.62
-  Louise pays Taylor: £98.96
-  Louise pays Jamie: £49.46
-  Klaus pays Jamie: £62.12
-  Klaus pays Sam: £71.58
-Please pay by bank transfer.
-Use your name as the reference.
+  Riley pays Alex: A$168.42
+  Quinn pays Alex: A$168.42
+  Jordan pays Alex: A$168.42
+  Dylan pays Alex: A$168.42
+  Drew pays Alex: A$117.90
+  Drew pays Morgan: A$50.52
+  Charlie pays Morgan: A$168.42
+  Blake pays Morgan: A$92.64
+  Blake pays Casey: A$75.78
+  Avery pays Casey: A$115.80
+  Avery pays Taylor: A$52.62
+  Louise pays Taylor: A$98.96
+  Louise pays Jamie: A$49.46
+  Klaus pays Jamie: A$62.12
+  Klaus pays Sam: A$71.58
+Please pay by bank transfer. Use your name as the reference.
 ─────────────────────────────────</t>
         </is>
       </c>
     </row>
+    <row r="42" ht="15" customHeight="1"/>
     <row r="43" ht="15" customHeight="1"/>
     <row r="44" ht="15" customHeight="1"/>
     <row r="45" ht="15" customHeight="1"/>
@@ -3244,10 +3701,9 @@
     <row r="79" ht="15" customHeight="1"/>
     <row r="80" ht="15" customHeight="1"/>
     <row r="81" ht="15" customHeight="1"/>
-    <row r="82" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B42:B82"/>
+    <mergeCell ref="B41:B81"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>